<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.003-07 Le cerceau jusqu'au chat
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.003-07.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.003-07.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>square, muret et gravier</t>
+          <t>square, portail, gravier, cerceau bleu, banc, gourde, fourmi</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raphaël, Mila, papa</t>
+          <t>Raphaël, Mila, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël veut que le cerceau bleu roule jusqu'au muret du chat, sans tomber. Une pierre arrête le cerceau. Mila l'écarte. Le chat ouvre un œil.</t>
+          <t>Le portail s'ouvre. Le fer grince. Sur le fer, un éclat de portail brille. Raphaël veut le cerceau bleu jusqu'au chat, maintenant. Mila arrive. Un rire commence. Mila se tait. Le cerceau tape la gourde. Raphaël refuse de foncer. Merci vécu. La queue du chat tombe. Il refuse, lit l'éclat. Un éclat de portail tient sur le fer.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un chat gris dort sur le muret du square. Sa queue pend un peu. Un volet orange claque tout doux. Le gravier crisse sous les semelles. Un cerceau bleu attend contre le banc. Le plastique est lisse et frais. Une feuille sèche tourne sur le gravier. Tu as vu le chat, Raphaël ? Il dort. Oui. Tout rond sur la pierre. Raphaël s'approche tout doux. Le chat ne bouge pas. Il ronronne ? Un tout petit peu. En ce moment, Raphaël tient le cerceau. Le plastique est un peu froid. Je veux qu'il aille au muret. Sans tomber. Jusqu'au chat ? Oui. Tout droit sur le gravier. Mila arrive près du banc. Ses pas font criss sur le gravier. Mila a des lunettes. Mila a les cheveux bouclés. Elle porte un gilet bleu. Mila, tu rattrapes au muret. Tu m'aides, Mila ? Oui. Raphaël pousse le cerceau. Il part tout droit. Le gravier crisse. Une petite poussière monte. Une pierre est sur le chemin. Le cerceau tape la pierre. Il tombe à plat. Le plastique fait un toc mou. Oh. On peut enlever la pierre. Pour ouvrir le chemin.</t>
+          <t>Le portail s'ouvre, un peu. Le fer grince, sec et long. Ça grince, papa ! Tu l'entends, le fer ? Oui, un petit cri. Sur le fer, un éclat de portail brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La gourde tape le bois du banc. Elle fait toc, rond et sourd. J'ai entendu le toc. La gourde, Raphaël ? Oui, papa. Le plastique est lisse, sous la main. Il est un peu froid. Une fourmi avance sur le gravier. Le gravier fait criss, sous ses pattes. Elle est petite. Tu la vois, la fourmi ? Oui, papa. En ce moment, Raphaël tient le cerceau. Le plastique bleu est un peu froid. Je veux qu'il aille au muret. Sans tomber, maintenant ! Jusqu'au chat ? Oui, papa. Tout droit, sur le gravier ? Oui, tout droit. Un chat gris dort sur le muret. Sa queue pend un peu. Il dort. Tout rond, Raphaël ? Oui. Mila arrive près du banc. Ses pas font criss sur le gravier. Mila a des lunettes. Mila a les cheveux bouclés. Elle porte un gilet bleu. Mila, tu rattrapes au muret ? Tu m'aides, Mila ? Oui. Raphaël regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Mila ne dit rien. Le sourire de Mila disparaît. Tu vas au muret, maintenant ! Mila recule d'un pas. Non. Oh. Raphaël pousse le cerceau trop vite, tout seul. Le cerceau tape la gourde. Il tombe à plat. Le plastique fait un toc mou. Il ne va pas ! La gourde est là. L'éclat de portail tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Mila, Raphaël ? Oui, papa. Tes mains sont froides, Raphaël ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un chat gris dort sur le muret du square. Sa queue pend un peu. Un volet orange claque tout doux. Le gravier crisse sous les semelles. Un cerceau bleu attend contre le banc. Le plastique est lisse et frais. Une feuille sèche tourne sur le gravier. Tu as vu le chat, Raphaël ? Il dort. Oui. Tout rond sur la pierre. Raphaël s'approche tout doux. Le chat ne bouge pas. Il ronronne ? Un tout petit peu. En ce moment, Raphaël tient le cerceau. Le plastique est un peu froid. Je veux qu'il aille au muret. Sans tomber. Jusqu'au chat ? Oui. Tout droit sur le gravier. Mila arrive près du banc. Ses pas font criss sur le gravier. Mila a des lunettes. Mila a les cheveux bouclés. Elle porte un gilet bleu. Mila, tu rattrapes au muret. Tu m'aides, Mila ? Oui. Raphaël pousse le cerceau. Il part tout droit. Le gravier crisse. Une petite poussière monte. Une pierre est sur le chemin. Le cerceau tape la pierre. Il tombe à plat. Le plastique fait un toc mou. Oh. On peut enlever la pierre. Pour ouvrir le chemin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le portail s'ouvre, un peu. Le fer grince, sec et long. Ça grince, papa ! Tu l'entends, le fer ? Oui, un petit cri. Sur le fer, un &lt;emphasis level="moderate"&gt;éclat de portail&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La gourde tape le bois du banc. Elle fait toc, rond et sourd. J'ai entendu le toc. La gourde, Raphaël ? Oui, papa. Le plastique est lisse, sous la main. Il est un peu froid. Une fourmi avance sur le gravier. Le gravier fait criss, sous ses pattes. Elle est petite. Tu la vois, la fourmi ? Oui, papa. En ce moment, Raphaël tient le cerceau. Le plastique bleu est un peu froid. Je veux qu'il aille au muret. Sans tomber, maintenant ! Jusqu'au chat ? Oui, papa. Tout droit, sur le gravier ? Oui, tout droit. Un chat gris dort sur le muret. Sa queue pend un peu. Il dort. Tout rond, Raphaël ? Oui. Mila arrive près du banc. Ses pas font criss sur le gravier. Mila a des lunettes. Mila a les cheveux bouclés. Elle porte un gilet bleu. Mila, tu rattrapes au muret ? Tu m'aides, Mila ? Oui. Raphaël regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Mila ne dit rien. Le sourire de Mila disparaît. Tu vas au muret, maintenant ! Mila recule d'un pas. Non. Oh. Raphaël pousse le cerceau trop vite, tout seul. Le cerceau tape la gourde. Il tombe à plat. Le plastique fait un toc mou. Il ne va pas ! La gourde est là. L'éclat de portail tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Mila, Raphaël ? Oui, papa. Tes mains sont froides, Raphaël ? Un peu, maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le matin, maman accompagne Éléonore au square. Un camarade arrive. Il a des lunettes. Il a les cheveux bouclés. Il porte un gilet bleu. Éléonore regarde. Un autre enfant laisse sortir un petit rire. Maman s'approche tout de suite. Maman dit : on ne va &lt;emphasis&gt;pas&lt;/emphasis&gt; rire de l'apparence. Les lunettes aident à voir. Les cheveux sont les cheveux. L'habit tient chaud. On joue. Éléonore hoche la tête. Elle va vers le camarade. Éléonore dit : tu viens aux cerceaux. Ils font rouler un cerceau. Plus tard, près du bac, un enfant regarde encore les lunettes. Éléonore dit : on ne va pas rire. On joue. On ne rit pas des lunettes, des cheveux ou d'un habit. On ne va pas rire de l'apparence. On joue ensemble. [pause]</t>
+          <t>Le portail s'ouvre, un peu. Le fer grince, sec et long. Ça grince, papa ! Tu l'entends, le fer ? Oui, un petit cri. Sur le fer, un &lt;emphasis&gt;éclat de portail&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La gourde tape le bois du banc. Elle fait toc, rond et sourd. J'ai entendu le toc. La gourde, Raphaël ? Oui, papa. Le plastique est lisse, sous la main. Il est un peu froid. Une fourmi avance sur le gravier. Le gravier fait criss, sous ses pattes. Elle est petite. Tu la vois, la fourmi ? Oui, papa. En ce moment, Raphaël tient le cerceau. Le plastique bleu est un peu froid. Je veux qu'il aille au muret. Sans tomber, maintenant ! Jusqu'au chat ? Oui, papa. Tout droit, sur le gravier ? Oui, tout droit. Un chat gris dort sur le muret. Sa queue pend un peu. Il dort. Tout rond, Raphaël ? Oui. Mila arrive près du banc. Ses pas font criss sur le gravier. Mila a des lunettes. Mila a les cheveux bouclés. Elle porte un gilet bleu. Mila, tu rattrapes au muret ? Tu m'aides, Mila ? Oui. Raphaël regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Mila ne dit rien. Le sourire de Mila disparaît. Tu vas au muret, maintenant ! Mila recule d'un pas. Non. Oh. Raphaël pousse le cerceau trop vite, tout seul. Le cerceau tape la gourde. Il tombe à plat. Le plastique fait un toc mou. Il ne va pas ! La gourde est là. L'éclat de portail tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Mila, Raphaël ? Oui, papa. Tes mains sont froides, Raphaël ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>éclat de portail</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,50 +1321,78 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_cerceau_jusqu_au_chat; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un chat gris dort sur le muret du square.
+          <t>narrateur|Le portail s'ouvre, un peu.
+narrateur|Le fer grince, sec et long.
+enfant-m|Ça grince, papa !
+papa|Tu l'entends, le fer ?
+enfant-m|Oui, un petit cri.
+narrateur|Sur le fer, un éclat de portail brille.
+enfant-m|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-m|Oui, un petit point.
+narrateur|La gourde tape le bois du banc.
+narrateur|Elle fait toc, rond et sourd.
+enfant-m|J'ai entendu le toc.
+papa|La gourde, Raphaël ?
+enfant-m|Oui, papa.
+maman|Le plastique est lisse, sous la main.
+enfant-m|Il est un peu froid.
+narrateur|Une fourmi avance sur le gravier.
+narrateur|Le gravier fait criss, sous ses pattes.
+enfant-m|Elle est petite.
+papa|Tu la vois, la fourmi ?
+enfant-m|Oui, papa.
+narrateur|En ce moment, Raphaël tient le cerceau.
+narrateur|Le plastique bleu est un peu froid.
+enfant-m|Je veux qu'il aille au muret.
+enfant-m|Sans tomber, maintenant !
+papa|Jusqu'au chat ?
+enfant-m|Oui, papa.
+maman|Tout droit, sur le gravier ?
+enfant-m|Oui, tout droit.
+narrateur|Un chat gris dort sur le muret.
 narrateur|Sa queue pend un peu.
-narrateur|Un volet orange claque tout doux.
-narrateur|Le gravier crisse sous les semelles.
-narrateur|Un cerceau bleu attend contre le banc.
-narrateur|Le plastique est lisse et frais.
-narrateur|Une feuille sèche tourne sur le gravier.
-papa|Tu as vu le chat, Raphaël ?
 enfant-m|Il dort.
-papa|Oui.
-papa|Tout rond sur la pierre.
-narrateur|Raphaël s'approche tout doux.
-narrateur|Le chat ne bouge pas.
-enfant-m|Il ronronne ?
-papa|Un tout petit peu.
-narrateur|En ce moment, Raphaël tient le cerceau.
-narrateur|Le plastique est un peu froid.
-enfant-m|Je veux qu'il aille au muret.
-enfant-m|Sans tomber.
-papa|Jusqu'au chat ?
+papa|Tout rond, Raphaël ?
 enfant-m|Oui.
-papa|Tout droit sur le gravier.
 narrateur|Mila arrive près du banc.
 narrateur|Ses pas font criss sur le gravier.
 narrateur|Mila a des lunettes.
 narrateur|Mila a les cheveux bouclés.
 narrateur|Elle porte un gilet bleu.
-papa|Mila, tu rattrapes au muret.
+papa|Mila, tu rattrapes au muret ?
 enfant-m|Tu m'aides, Mila ?
 copine|Oui.
-narrateur|Raphaël pousse le cerceau.
-narrateur|Il part tout droit.
-narrateur|Le gravier crisse.
-narrateur|Une petite poussière monte.
-narrateur|Une pierre est sur le chemin.
-narrateur|Le cerceau tape la pierre.
+narrateur|Raphaël regarde les lunettes, trop longtemps.
+narrateur|Un rire commence dans sa bouche.
+narrateur|Mila ne dit rien.
+narrateur|Le sourire de Mila disparaît.
+enfant-m|Tu vas au muret, maintenant !
+narrateur|Mila recule d'un pas.
+copine|Non.
+enfant-m|Oh.
+narrateur|Raphaël pousse le cerceau trop vite, tout seul.
+narrateur|Le cerceau tape la gourde.
 narrateur|Il tombe à plat.
 narrateur|Le plastique fait un toc mou.
-enfant-m|Oh.
-papa|On peut enlever la pierre.
-papa|Pour ouvrir le chemin.</t>
+enfant-m|Il ne va pas !
+copine|La gourde est là.
+narrateur|L'éclat de portail tremble, puis tient.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Mila, Raphaël ?
+enfant-m|Oui, papa.
+maman|Tes mains sont froides, Raphaël ?
+enfant-m|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1401,22 +1429,22 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila a des lunettes. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila a des &lt;emphasis level="moderate"&gt;lunettes&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le camarade a des lunettes. Que fait-on ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila a des &lt;emphasis&gt;lunettes&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>jouer</t>
+          <t>pas rire</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>jouer | ensemble | pierre | cerceau | on joue | pas rire</t>
+          <t>pas rire | on joue | jouer | pas rire apparence</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1431,7 +1459,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On ôte la pierre. Que fait-on ?</t>
+          <t>Pas rire. Mila a des lunettes. Que fait-on ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1469,7 +1497,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1480,7 +1508,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1495,34 +1523,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>lunettes</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1537,17 +1569,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=mila_a_des_lunettes_pas_rire; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1580,17 +1612,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila se penche. Elle voit la pierre grise. La pierre est là. Raphaël l'écarte avec le pied. La pierre roule vers l'herbe. Merci, Raphaël. Merci, Mila. Mila a vu la pierre. Le chemin est libre. On reprend ? On reprend. Raphaël pose le cerceau. Mila attend près du muret. Tu le rattrapes, Mila. Je suis prête.</t>
+          <t>Raphaël veut le cerceau au muret, tout de suite. Je pousse, maintenant ! Il avance trop vite vers Mila. Les mots se bousculent dans sa bouche. Non. Mila reste un peu plus loin. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le cerceau, un instant. Il écoute le grincement du portail. Tu veux le cerceau avec Mila ? Papa reste à la même hauteur. Tu rattrapes au muret ? Mila ne dit rien, d'abord. Elle pose les mains près du plastique. Je le tiens. D'accord. Merci, Raphaël. Papa a vu les deux, près du banc. La gourde a bougé, sous le cerceau. Elle est tombée. Ils écartent la gourde du chemin. Mila tient le plastique, plus près. Le cerceau redevient plus léger, cette fois. Il tient ! Oui. Tu le vois, le cerceau ? Oui, papa. Au muret, Mila ? J'y vais. Raphaël pousse, sans se presser. Mila suit le plastique des yeux. Le cerceau avance un peu. Il roule. Il roule. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près du banc ? Oui. Tes mains sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila se penche. Elle voit la pierre grise. La pierre est là. Raphaël l'écarte avec le pied. La pierre roule vers l'herbe. Merci, Raphaël. Merci, Mila. Mila a vu la pierre. Le chemin est libre. On reprend ? On reprend. Raphaël pose le cerceau. Mila attend près du muret. Tu le rattrapes, Mila. Je suis prête.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël veut le &lt;emphasis level="moderate"&gt;cerceau&lt;/emphasis&gt; au muret, tout de suite. Je pousse, maintenant ! Il avance trop vite vers Mila. Les mots se bousculent dans sa bouche. Non. Mila reste un peu plus loin. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le cerceau, un instant. Il écoute le grincement du portail. Tu veux le cerceau avec Mila ? Papa reste à la même hauteur. Tu rattrapes au muret ? Mila ne dit rien, d'abord. Elle pose les mains près du plastique. Je le tiens. D'accord. Merci, Raphaël. Papa a vu les deux, près du banc. La gourde a bougé, sous le cerceau. Elle est tombée. Ils écartent la gourde du chemin. Mila tient le plastique, plus près. Le cerceau redevient plus léger, cette fois. Il tient ! Oui. Tu le vois, le cerceau ? Oui, papa. Au muret, Mila ? J'y vais. Raphaël pousse, sans se presser. Mila suit le plastique des yeux. Le cerceau avance un peu. Il roule. Il roule. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près du banc ? Oui. Tes mains sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Éléonore a entendu maman. On ne va &lt;emphasis&gt;pas&lt;/emphasis&gt; rire de l'apparence. Elle a joué avec le camarade. [pause]</t>
+          <t>Raphaël veut le &lt;emphasis&gt;cerceau&lt;/emphasis&gt; au muret, tout de suite. Je pousse, maintenant ! Il avance trop vite vers Mila. Les mots se bousculent dans sa bouche. Non. Mila reste un peu plus loin. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le cerceau, un instant. Il écoute le grincement du portail. Tu veux le cerceau avec Mila ? Papa reste à la même hauteur. Tu rattrapes au muret ? Mila ne dit rien, d'abord. Elle pose les mains près du plastique. Je le tiens. D'accord. Merci, Raphaël. Papa a vu les deux, près du banc. La gourde a bougé, sous le cerceau. Elle est tombée. Ils écartent la gourde du chemin. Mila tient le plastique, plus près. Le cerceau redevient plus léger, cette fois. Il tient ! Oui. Tu le vois, le cerceau ? Oui, papa. Au muret, Mila ? J'y vais. Raphaël pousse, sans se presser. Mila suit le plastique des yeux. Le cerceau avance un peu. Il roule. Il roule. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près du banc ? Oui. Tes mains sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1637,7 +1669,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1645,10 +1677,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1671,30 +1703,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>cerceau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1703,10 +1735,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1719,26 +1751,60 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=ils_tiennent_le_cerceau_a_deux; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila se penche.
-narrateur|Elle voit la pierre grise.
-copine|La pierre est là.
-narrateur|Raphaël l'écarte avec le pied.
-narrateur|La pierre roule vers l'herbe.
+          <t>narrateur|Raphaël veut le cerceau au muret, tout de suite.
+enfant-m|Je pousse, maintenant !
+narrateur|Il avance trop vite vers Mila.
+narrateur|Les mots se bousculent dans sa bouche.
+copine|Non.
+narrateur|Mila reste un peu plus loin.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe le cerceau, un instant.
+narrateur|Il écoute le grincement du portail.
+papa|Tu veux le cerceau avec Mila ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Tu rattrapes au muret ?
+narrateur|Mila ne dit rien, d'abord.
+narrateur|Elle pose les mains près du plastique.
+copine|Je le tiens.
+enfant-m|D'accord.
 papa|Merci, Raphaël.
-papa|Merci, Mila.
-papa|Mila a vu la pierre.
-papa|Le chemin est libre.
-enfant-m|On reprend ?
-copine|On reprend.
-narrateur|Raphaël pose le cerceau.
-narrateur|Mila attend près du muret.
-papa|Tu le rattrapes, Mila.
-copine|Je suis prête.</t>
+narrateur|Papa a vu les deux, près du banc.
+maman|La gourde a bougé, sous le cerceau.
+enfant-m|Elle est tombée.
+narrateur|Ils écartent la gourde du chemin.
+narrateur|Mila tient le plastique, plus près.
+narrateur|Le cerceau redevient plus léger, cette fois.
+enfant-m|Il tient !
+copine|Oui.
+papa|Tu le vois, le cerceau ?
+enfant-m|Oui, papa.
+maman|Au muret, Mila ?
+copine|J'y vais.
+narrateur|Raphaël pousse, sans se presser.
+narrateur|Mila suit le plastique des yeux.
+narrateur|Le cerceau avance un peu.
+copine|Il roule.
+enfant-m|Il roule.
+narrateur|Le ventre de Raphaël se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près du banc ?
+enfant-m|Oui.
+maman|Tes mains sont au chaud ?
+enfant-m|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>cerceau</t>
         </is>
       </c>
     </row>
@@ -1765,17 +1831,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Le cerceau bleu roule encore. Le chemin est libre. Il avance, il avance. Le plastique chante un peu. Il arrive au muret. Je l'ai ! Il n'est pas tombé. Bravo. Vous avez ôté la pierre. Le chat ouvre un œil. Ses moustaches bougent un peu. Il nous a vus. Puis il se rendort. Le volet claque encore un peu. On le ramène au banc ? Doucement. Mila fait rouler le cerceau. Raphaël le rattrape. Le plastique tape le bois. Toc. Oui. Il est rentré. Le chat a ouvert un œil. Puis il a dormi.</t>
+          <t>Le cerceau roule, plus vite. Il avance. Jusqu'au chat, maintenant ! Le gilet bleu bouge. Les boucles tapent le dos. Les lunettes restent sur le nez. Le chat ouvre un œil. Sa queue tombe sur le gravier. Il passe, maintenant ! Il pousse trop vite, tout de suite. Il regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Mila lâche le plastique. Le cerceau penche vers la queue. Ça tombe ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le cerceau, un instant. Il écoute le grincement du portail. Sur le fer, un éclat de portail luit. Là, sur le fer. Tu rattrapes, Mila ? Mila ne dit rien. Elle reprend le plastique, sans parler. Oui. Ils attendent un peu. Le chat rentre sa queue. Raphaël pousse, sans se presser. Mila rattrape. Je l'ai ! Il n'est pas tombé. Tu as poussé sans t'arrêter ? Oui, papa. Le gilet est chaud, Mila ? Un peu. Le cerceau se pose contre le muret. On reverse les rôles ? À toi le muret. Mila pousse à son tour. Raphaël rattrape. Le plastique tape le bois. Toc. Le cerceau est arrivé ? Oui, papa. Un rayon passe sur le fer. Il allume le gilet.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Le cerceau bleu roule encore. Le chemin est libre. Il avance, il avance. Le plastique chante un peu. Il arrive au muret. Je l'ai ! Il n'est pas tombé. Bravo. Vous avez ôté la pierre. Le chat ouvre un œil. Ses moustaches bougent un peu. Il nous a vus. Puis il se rendort. Le volet claque encore un peu. On le ramène au banc ? Doucement. Mila fait rouler le cerceau. Raphaël le rattrape. Le plastique tape le bois. Toc. Oui. Il est rentré. Le chat a ouvert un œil. Puis il a dormi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cerceau roule, plus vite. Il avance. Jusqu'au chat, maintenant ! Le gilet bleu bouge. Les boucles tapent le dos. Les lunettes restent sur le nez. Le chat ouvre un œil. Sa queue tombe sur le gravier. Il passe, maintenant ! Il pousse trop vite, tout de suite. Il regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Mila lâche le plastique. Le cerceau penche vers la queue. Ça tombe ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le cerceau, un instant. Il écoute le grincement du portail. Sur le fer, un &lt;emphasis level="moderate"&gt;éclat de portail&lt;/emphasis&gt; luit. Là, sur le fer. Tu rattrapes, Mila ? Mila ne dit rien. Elle reprend le plastique, sans parler. Oui. Ils attendent un peu. Le chat rentre sa queue. Raphaël pousse, sans se presser. Mila rattrape. Je l'ai ! Il n'est pas tombé. Tu as poussé sans t'arrêter ? Oui, papa. Le gilet est chaud, Mila ? Un peu. Le cerceau se pose contre le muret. On reverse les rôles ? À toi le muret. Mila pousse à son tour. Raphaël rattrape. Le plastique tape le bois. Toc. Le cerceau est arrivé ? Oui, papa. Un rayon passe sur le fer. Il allume le gilet.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman revient près du portail. Éléonore et le camarade se disent à de&lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Le cerceau roule, plus vite. Il avance. Jusqu'au chat, maintenant ! Le gilet bleu bouge. Les boucles tapent le dos. Les lunettes restent sur le nez. Le chat ouvre un œil. Sa queue tombe sur le gravier. Il passe, maintenant ! Il pousse trop vite, tout de suite. Il regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Mila lâche le plastique. Le cerceau penche vers la queue. Ça tombe ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le cerceau, un instant. Il écoute le grincement du portail. Sur le fer, un &lt;emphasis&gt;éclat de portail&lt;/emphasis&gt; luit. Là, sur le fer. Tu rattrapes, Mila ? Mila ne dit rien. Elle reprend le plastique, sans parler. Oui. Ils attendent un peu. Le chat rentre sa queue. Raphaël pousse, sans se presser. Mila rattrape. Je l'ai ! Il n'est pas tombé. Tu as poussé sans t'arrêter ? Oui, papa. Le gilet est chaud, Mila ? Un peu. Le cerceau se pose contre le muret. On reverse les rôles ? À toi le muret. Mila pousse à son tour. Raphaël rattrape. Le plastique tape le bois. Toc. Le cerceau est arrivé ? Oui, papa. Un rayon passe sur le fer. Il allume le gilet. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1822,7 +1888,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1830,10 +1896,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1856,30 +1922,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de portail</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1888,10 +1954,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1902,33 +1968,68 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Le cerceau bleu roule encore.
-narrateur|Le chemin est libre.
-narrateur|Il avance, il avance.
-narrateur|Le plastique chante un peu.
-narrateur|Il arrive au muret.
+          <t>narrateur|Le cerceau roule, plus vite.
+copine|Il avance.
+enfant-m|Jusqu'au chat, maintenant !
+narrateur|Le gilet bleu bouge.
+narrateur|Les boucles tapent le dos.
+narrateur|Les lunettes restent sur le nez.
+narrateur|Le chat ouvre un œil.
+narrateur|Sa queue tombe sur le gravier.
+enfant-m|Il passe, maintenant !
+narrateur|Il pousse trop vite, tout de suite.
+narrateur|Il regarde les lunettes, trop longtemps.
+narrateur|Un rire revient dans sa bouche.
+copine|Attends.
+narrateur|Mila lâche le plastique.
+narrateur|Le cerceau penche vers la queue.
+enfant-m|Ça tombe !
+narrateur|Raphaël avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Raphaël refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le cerceau, un instant.
+narrateur|Il écoute le grincement du portail.
+narrateur|Sur le fer, un éclat de portail luit.
+enfant-m|Là, sur le fer.
+enfant-m|Tu rattrapes, Mila ?
+narrateur|Mila ne dit rien.
+narrateur|Elle reprend le plastique, sans parler.
+copine|Oui.
+narrateur|Ils attendent un peu.
+narrateur|Le chat rentre sa queue.
+narrateur|Raphaël pousse, sans se presser.
+narrateur|Mila rattrape.
 copine|Je l'ai !
 enfant-m|Il n'est pas tombé.
-papa|Bravo.
-papa|Vous avez ôté la pierre.
-narrateur|Le chat ouvre un œil.
-narrateur|Ses moustaches bougent un peu.
-enfant-m|Il nous a vus.
-papa|Puis il se rendort.
-narrateur|Le volet claque encore un peu.
-papa|On le ramène au banc ?
-enfant-m|Doucement.
-narrateur|Mila fait rouler le cerceau.
-narrateur|Raphaël le rattrape.
+papa|Tu as poussé sans t'arrêter ?
+enfant-m|Oui, papa.
+maman|Le gilet est chaud, Mila ?
+copine|Un peu.
+narrateur|Le cerceau se pose contre le muret.
+papa|On reverse les rôles ?
+copine|À toi le muret.
+narrateur|Mila pousse à son tour.
+narrateur|Raphaël rattrape.
 narrateur|Le plastique tape le bois.
 enfant-m|Toc.
-papa|Oui.
-papa|Il est rentré.
-copine|Le chat a ouvert un œil.
-enfant-m|Puis il a dormi.</t>
+papa|Le cerceau est arrivé ?
+enfant-m|Oui, papa.
+maman|Un rayon passe sur le fer.
+enfant-m|Il allume le gilet.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>cerceau</t>
         </is>
       </c>
     </row>
@@ -1955,17 +2056,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le cerceau bleu repose contre le banc. Le chat dort encore sur le muret. Il est allé jusqu'au chat. Oui. Vous avez ôté la pierre. Le gravier redevient calme.</t>
+          <t>Ils restent près du banc. Maman essuie un peu de gravier. On a eu le cerceau, papa. Tu l'as vu, toi ? Oui, au muret. On est bien, ici. Raphaël tapote le plastique du doigt. Il a une trace de gourde. Tu la vois, la trace ? Oui, maman. Le cerceau est resté, Raphaël. Oui, avec Mila. Le cerceau est resté. Ça sent le fer, un peu tiède. Et le portail, maman. Oui, dans l'air. La fourmi reste sur le gravier. Un éclat de portail tient sur le fer.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le cerceau bleu repose contre le banc. Le chat dort encore sur le muret. Il est allé jusqu'au chat. Oui. Vous avez ôté la pierre. Le gravier redevient calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du banc. Maman essuie un peu de gravier. On a eu le cerceau, papa. Tu l'as vu, toi ? Oui, au muret. On est bien, ici. Raphaël tapote le plastique du doigt. Il a une trace de gourde. Tu la vois, la trace ? Oui, maman. Le cerceau est resté, Raphaël. Oui, avec Mila. Le cerceau est resté. Ça sent le fer, un peu tiède. Et le portail, maman. Oui, dans l'air. La fourmi reste sur le gravier. Un &lt;emphasis level="moderate"&gt;éclat de portail&lt;/emphasis&gt; tient sur le fer.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du banc. Maman essuie un peu de gravier. On a eu le cerceau, papa. Tu l'as vu, toi ? Oui, au muret. On est bien, ici. Raphaël tapote le plastique du doigt. Il a une trace de gourde. Tu la vois, la trace ? Oui, maman. Le cerceau est resté, Raphaël. Oui, avec Mila. Le cerceau est resté. Ça sent le fer, un peu tiède. Et le portail, maman. Oui, dans l'air. La fourmi reste sur le gravier. Un &lt;emphasis&gt;éclat de portail&lt;/emphasis&gt; tient sur le fer.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2012,18 +2113,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2032,12 +2133,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2046,17 +2147,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de portail</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2065,11 +2170,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2078,29 +2183,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_fer; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le cerceau bleu repose contre le banc.
-narrateur|Le chat dort encore sur le muret.
-enfant-m|Il est allé jusqu'au chat.
-papa|Oui.
-papa|Vous avez ôté la pierre.
-narrateur|Le gravier redevient calme.</t>
+          <t>narrateur|Ils restent près du banc.
+narrateur|Maman essuie un peu de gravier.
+enfant-m|On a eu le cerceau, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, au muret.
+maman|On est bien, ici.
+narrateur|Raphaël tapote le plastique du doigt.
+enfant-m|Il a une trace de gourde.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le cerceau est resté, Raphaël.
+enfant-m|Oui, avec Mila.
+copine|Le cerceau est resté.
+narrateur|Ça sent le fer, un peu tiède.
+enfant-m|Et le portail, maman.
+maman|Oui, dans l'air.
+narrateur|La fourmi reste sur le gravier.
+narrateur|Un éclat de portail tient sur le fer.</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2206,6 +2327,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>